<commit_message>
fixed issues in emanating and pr
</commit_message>
<xml_diff>
--- a/docs/6. emanating-template.xlsx
+++ b/docs/6. emanating-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Patriach\Downloads\laravel\procurex\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3485D202-84CA-4352-A372-83D85EB8B448}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6B6CBB5-BA99-4017-877D-BF4090D026A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,25 +57,13 @@
     <t>PARTICULARS/ ITEM/DESCRIPTION</t>
   </si>
   <si>
-    <t>20 pcs</t>
-  </si>
-  <si>
     <t>Training Kit</t>
   </si>
   <si>
-    <t>3 persons</t>
-  </si>
-  <si>
     <t>Honorarium for Resource Person</t>
   </si>
   <si>
-    <t>50 pax</t>
-  </si>
-  <si>
     <t>Meals &amp; Snacks (AM Snacks &amp; Lunch)</t>
-  </si>
-  <si>
-    <t>60 pcs</t>
   </si>
   <si>
     <t>Tshirt with collar and print premium dry fit</t>
@@ -164,6 +152,18 @@
       </rPr>
       <t>3rd</t>
     </r>
+  </si>
+  <si>
+    <t>10 pcs</t>
+  </si>
+  <si>
+    <t>2 persons</t>
+  </si>
+  <si>
+    <t>30 pax</t>
+  </si>
+  <si>
+    <t>30 pcs</t>
   </si>
 </sst>
 </file>
@@ -357,19 +357,19 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -741,17 +741,17 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B1" s="2" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="16.5" x14ac:dyDescent="0.3">
@@ -760,25 +760,25 @@
       <c r="C5" s="1"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="19"/>
-      <c r="C6" s="19"/>
+      <c r="B6" s="22"/>
+      <c r="C6" s="22"/>
     </row>
     <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A7" s="20" t="s">
+      <c r="A7" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="19"/>
-      <c r="C7" s="19"/>
+      <c r="B7" s="22"/>
+      <c r="C7" s="22"/>
     </row>
     <row r="8" spans="1:3" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A8" s="20" t="s">
+      <c r="A8" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="B8" s="19"/>
-      <c r="C8" s="19"/>
+      <c r="B8" s="22"/>
+      <c r="C8" s="22"/>
     </row>
     <row r="9" spans="1:3" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -824,13 +824,13 @@
       <c r="B16" s="2"/>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="21" t="s">
-        <v>31</v>
+      <c r="A17" s="18" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="21" t="s">
-        <v>30</v>
+      <c r="A18" s="18" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -847,34 +847,34 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" s="6" t="s">
         <v>10</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="16.5" x14ac:dyDescent="0.25">
@@ -963,41 +963,41 @@
     </row>
     <row r="46" spans="1:2" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A46" s="14" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B46" s="15" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A47" s="22" t="s">
-        <v>20</v>
-      </c>
-      <c r="B47" s="23" t="s">
-        <v>21</v>
+      <c r="A47" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="B47" s="20" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B48" s="15" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
     </row>
     <row r="51" spans="2:2" ht="33" x14ac:dyDescent="0.25">
       <c r="B51" s="17" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
     </row>
     <row r="52" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B52" s="16" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
     </row>
     <row r="53" spans="2:2" ht="16.5" x14ac:dyDescent="0.25">
       <c r="B53" s="15" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>